<commit_message>
Improvments för tests and mail ok
</commit_message>
<xml_diff>
--- a/examples/brakform_4_rakn_3_nivaer.xlsx
+++ b/examples/brakform_4_rakn_3_nivaer.xlsx
@@ -505,7 +505,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B5" t="str">
         <v>single_choice</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B9" t="str">
         <v>single_choice</v>
@@ -713,7 +713,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B13" t="str">
         <v>single_choice</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B17" t="str">
         <v>single_choice</v>
@@ -921,7 +921,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B21" t="str">
         <v>single_choice</v>
@@ -1025,7 +1025,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B25" t="str">
         <v>single_choice</v>
@@ -1129,7 +1129,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B29" t="str">
         <v>single_choice</v>
@@ -1233,7 +1233,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B33" t="str">
         <v>single_choice</v>
@@ -1337,7 +1337,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B37" t="str">
         <v>single_choice</v>
@@ -1441,7 +1441,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B41" t="str">
         <v>single_choice</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>$\frac{5}{6} \div \frac{1}{3}$</v>
+        <v>$\frac{5}{6} / \frac{1}{3}$</v>
       </c>
       <c r="B45" t="str">
         <v>single_choice</v>
@@ -1649,7 +1649,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{5}$</v>
+        <v>$\frac{9}{10} / \frac{3}{5}$</v>
       </c>
       <c r="B49" t="str">
         <v>single_choice</v>
@@ -1805,7 +1805,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>$\frac{7}{8} \div \frac{1}{2}$</v>
+        <v>$\frac{7}{8} / \frac{1}{2}$</v>
       </c>
       <c r="B55" t="str">
         <v>single_choice</v>
@@ -1909,7 +1909,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{4}$</v>
+        <v>$\frac{9}{10} / \frac{3}{4}$</v>
       </c>
       <c r="B59" t="str">
         <v>single_choice</v>
@@ -2013,7 +2013,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>$\frac{7}{8} \div \frac{1}{2}$</v>
+        <v>$\frac{7}{8} / \frac{1}{2}$</v>
       </c>
       <c r="B63" t="str">
         <v>single_choice</v>
@@ -2117,7 +2117,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{4}$</v>
+        <v>$\frac{9}{10} / \frac{3}{4}$</v>
       </c>
       <c r="B67" t="str">
         <v>single_choice</v>
@@ -2221,7 +2221,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>$\frac{7}{8} \div \frac{1}{2}$</v>
+        <v>$\frac{7}{8} / \frac{1}{2}$</v>
       </c>
       <c r="B71" t="str">
         <v>single_choice</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>$\frac{9}{10} \div \frac{3}{4}$</v>
+        <v>$\frac{9}{10} / \frac{3}{4}$</v>
       </c>
       <c r="B75" t="str">
         <v>single_choice</v>
@@ -2429,7 +2429,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>$\frac{7}{8} \div \frac{1}{2}$</v>
+        <v>$\frac{7}{8} / \frac{1}{2}$</v>
       </c>
       <c r="B79" t="str">
         <v>single_choice</v>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) \div \frac{1}{2}$</v>
+        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) / \frac{1}{2}$</v>
       </c>
       <c r="B82" t="str">
         <v>single_choice</v>
@@ -2585,7 +2585,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) \div \frac{3}{4}$</v>
+        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) / \frac{3}{4}$</v>
       </c>
       <c r="B85" t="str">
         <v>single_choice</v>
@@ -2637,7 +2637,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>$\frac{3}{5} \cdot \frac{10}{9} \div \frac{2}{3}$</v>
+        <v>$\frac{3}{5} \cdot \frac{10}{9} / \frac{2}{3}$</v>
       </c>
       <c r="B87" t="str">
         <v>single_choice</v>
@@ -2663,7 +2663,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>$\left(\frac{5}{8} + \frac{3}{4}\right) \div \frac{1}{2}$</v>
+        <v>$\left(\frac{5}{8} + \frac{3}{4}\right) / \frac{1}{2}$</v>
       </c>
       <c r="B88" t="str">
         <v>single_choice</v>
@@ -2715,7 +2715,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) \div \frac{1}{2}$</v>
+        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) / \frac{1}{2}$</v>
       </c>
       <c r="B90" t="str">
         <v>single_choice</v>
@@ -2793,7 +2793,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) \div \frac{3}{4}$</v>
+        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) / \frac{3}{4}$</v>
       </c>
       <c r="B93" t="str">
         <v>single_choice</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>$\frac{3}{5} \cdot \frac{10}{9} \div \frac{2}{3}$</v>
+        <v>$\frac{3}{5} \cdot \frac{10}{9} / \frac{2}{3}$</v>
       </c>
       <c r="B95" t="str">
         <v>single_choice</v>
@@ -2871,7 +2871,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>$\left(\frac{5}{8} + \frac{3}{4}\right) \div \frac{1}{2}$</v>
+        <v>$\left(\frac{5}{8} + \frac{3}{4}\right) / \frac{1}{2}$</v>
       </c>
       <c r="B96" t="str">
         <v>single_choice</v>
@@ -2923,7 +2923,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) \div \frac{1}{2}$</v>
+        <v>$\left(\frac{2}{3} + \frac{1}{6}\right) / \frac{1}{2}$</v>
       </c>
       <c r="B98" t="str">
         <v>single_choice</v>
@@ -3001,7 +3001,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) \div \frac{3}{4}$</v>
+        <v>$\left(\frac{7}{8} - \frac{1}{4}\right) / \frac{3}{4}$</v>
       </c>
       <c r="B101" t="str">
         <v>single_choice</v>

</xml_diff>